<commit_message>
Keep battery recharge time normal
</commit_message>
<xml_diff>
--- a/LongSubmerged10x/Data Sheets/Entities.xlsx
+++ b/LongSubmerged10x/Data Sheets/Entities.xlsx
@@ -1029,7 +1029,7 @@
       </c>
       <c r="P8" s="8" t="inlineStr">
         <is>
-          <t>/Velocity +1, Noise = 0.7, FuelUsage = 1.0, EnergyUsage = -0.1, SmokeVisibility = 0.25, MaxGearChangeDelay = 7</t>
+          <t>/Velocity +1, Noise = 0.7, FuelUsage = 1.0, EnergyUsage = -10, SmokeVisibility = 0.25, MaxGearChangeDelay = 7</t>
         </is>
       </c>
       <c r="Q8" s="4" t="n"/>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
-          <t>/Velocity +1, Noise = 0.35, FuelUsage = 1.0, EnergyUsage = -0.1, SmokeVisibility = 0.25, MaxGearChangeDelay = 7</t>
+          <t>/Velocity +1, Noise = 0.35, FuelUsage = 1.0, EnergyUsage = -10, SmokeVisibility = 0.25, MaxGearChangeDelay = 7</t>
         </is>
       </c>
       <c r="Q9" s="4" t="n"/>

</xml_diff>

<commit_message>
Raise player submarine top speed cap
</commit_message>
<xml_diff>
--- a/LongSubmerged10x/Data Sheets/Entities.xlsx
+++ b/LongSubmerged10x/Data Sheets/Entities.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Types" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,8 +33,31 @@
       <name val="Calibri"/>
       <charset val="238"/>
       <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="238"/>
+      <family val="2"/>
       <b val="1"/>
       <color rgb="FF44546A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="238"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="238"/>
+      <family val="2"/>
+      <color rgb="FF006100"/>
       <sz val="11"/>
     </font>
     <font>
@@ -43,23 +67,22 @@
       <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="238"/>
-      <family val="2"/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFCCFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -81,6 +104,15 @@
       <right/>
       <top/>
       <bottom style="medium">
+        <color theme="4" tint="0.3999755851924192"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
         <color rgb="FF8FAADC"/>
       </bottom>
       <diagonal/>
@@ -89,30 +121,48 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="4"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="4"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -480,6 +530,547 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:V7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="39.54296875" customWidth="1" min="1" max="1"/>
+    <col width="24.453125" customWidth="1" min="2" max="2"/>
+    <col width="13.453125" customWidth="1" min="3" max="3"/>
+    <col width="10.453125" customWidth="1" min="4" max="4"/>
+    <col width="9.453125" customWidth="1" min="5" max="5"/>
+    <col width="9.54296875" customWidth="1" min="6" max="6"/>
+    <col width="8.54296875" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14.54296875" customWidth="1" min="9" max="9"/>
+    <col width="10.453125" customWidth="1" min="11" max="11"/>
+    <col width="8.453125" customWidth="1" min="12" max="12"/>
+    <col width="9.453125" customWidth="1" min="14" max="14"/>
+    <col width="13.54296875" customWidth="1" min="16" max="16"/>
+    <col width="22.453125" customWidth="1" min="18" max="18"/>
+    <col width="115.1796875" customWidth="1" min="19" max="19"/>
+    <col width="36.453125" customWidth="1" min="20" max="20"/>
+    <col width="43.54296875" customWidth="1" min="21" max="21"/>
+    <col width="19.54296875" customWidth="1" min="22" max="22"/>
+    <col width="8.54296875" customWidth="1" min="23" max="23"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Displacement (t)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+      <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="n"/>
+      <c r="O1" s="1" t="n"/>
+      <c r="P1" s="1" t="n"/>
+      <c r="Q1" s="1" t="n"/>
+      <c r="R1" s="1" t="n"/>
+      <c r="S1" s="1" t="n"/>
+      <c r="T1" s="1" t="n"/>
+      <c r="U1" s="1" t="n"/>
+      <c r="V1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Speed (km/h)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Length (m)</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Beam (m)</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Draught (m)</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Mast height (m)</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>GRT</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>Range (km)</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Crew</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Threat</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Military</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>Is Class</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>Reward</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>Iron Cross</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>Estimated Durability (AI)</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>Parameters</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="inlineStr">
+        <is>
+          <t>Prefab Path</t>
+        </is>
+      </c>
+      <c r="U2" s="4" t="inlineStr">
+        <is>
+          <t>Recognized As</t>
+        </is>
+      </c>
+      <c r="V2" s="1" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Type IIA (Player)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Submarine</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>769</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>871</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J3" s="7" t="n"/>
+      <c r="K3" s="5" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="M3" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="P3" s="1" t="n">
+        <v>7500</v>
+      </c>
+      <c r="Q3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="S3" s="8" t="inlineStr">
+        <is>
+          <t>Observation Spot/SightRange = 7500, Observation Spot/GroupSightRange = 13, AreaSize = 7.5, SpawnSpacing = 300, HullFrontalVisibilityFactor *= 0.65, HullBaseVisibilityFactor *= 0.58, IndirectVisualDetectability *= 0.55, UnderwaterFadeFactor *= 2.0, CrushDepth = -200, SonarDetectability *= 0.55</t>
+        </is>
+      </c>
+      <c r="T3" s="8" t="inlineStr">
+        <is>
+          <t>Entities/</t>
+        </is>
+      </c>
+      <c r="U3" s="1" t="n"/>
+      <c r="V3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Type IID (Player)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Submarine</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>769</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>871</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J4" s="7" t="n"/>
+      <c r="K4" s="5" t="n">
+        <v>10460</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="P4" s="1" t="n">
+        <v>7500</v>
+      </c>
+      <c r="Q4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="S4" s="8" t="inlineStr">
+        <is>
+          <t>Observation Spot/SightRange = 7500, Observation Spot/GroupSightRange = 13, AreaSize = 7.5, SpawnSpacing = 300, HullFrontalVisibilityFactor *= 0.65, HullBaseVisibilityFactor *= 0.58, IndirectVisualDetectability *= 0.55, UnderwaterFadeFactor *= 2.0, CrushDepth = -200, SonarDetectability *= 0.55</t>
+        </is>
+      </c>
+      <c r="T4" s="8" t="inlineStr">
+        <is>
+          <t>Entities/</t>
+        </is>
+      </c>
+      <c r="U4" s="1" t="n"/>
+      <c r="V4" s="1" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Type VIIB (Player)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Submarine</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>769</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>871</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J5" s="7" t="n"/>
+      <c r="K5" s="5" t="n">
+        <v>15700</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="P5" s="1" t="n">
+        <v>7500</v>
+      </c>
+      <c r="Q5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="S5" s="8" t="inlineStr">
+        <is>
+          <t>Observation Spot/SightRange = 8500, Observation Spot/GroupSightRange = 13, AreaSize = 7.5, SpawnSpacing = 300, HullFrontalVisibilityFactor *= 0.65, HullBaseVisibilityFactor *= 0.68, IndirectVisualDetectability *= 0.7, UnderwaterFadeFactor *= 2.0, CrushDepth = -250</t>
+        </is>
+      </c>
+      <c r="T5" s="8" t="inlineStr">
+        <is>
+          <t>Entities/</t>
+        </is>
+      </c>
+      <c r="U5" s="1" t="n"/>
+      <c r="V5" s="1" t="n"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Type VIIC (Player)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Submarine</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>769</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>871</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="5" t="n">
+        <v>15700</v>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="M6" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="P6" s="1" t="n">
+        <v>7500</v>
+      </c>
+      <c r="Q6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="S6" s="8" t="inlineStr">
+        <is>
+          <t>Observation Spot/SightRange = 8500, Observation Spot/GroupSightRange = 13, AreaSize = 7.5, SpawnSpacing = 300, HullFrontalVisibilityFactor *= 0.65, HullBaseVisibilityFactor *= 0.68, IndirectVisualDetectability *= 0.7, UnderwaterFadeFactor *= 2.0, CrushDepth = -250</t>
+        </is>
+      </c>
+      <c r="T6" s="8" t="inlineStr">
+        <is>
+          <t>Entities/</t>
+        </is>
+      </c>
+      <c r="U6" s="1" t="n"/>
+      <c r="V6" s="1" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Type VIIC41 (Player)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Submarine</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>769</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>871</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="5" t="n">
+        <v>15700</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="P7" s="1" t="n">
+        <v>7500</v>
+      </c>
+      <c r="Q7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="S7" s="8" t="inlineStr">
+        <is>
+          <t>Observation Spot/SightRange = 8500, Observation Spot/GroupSightRange = 13, AreaSize = 7.5, SpawnSpacing = 300, HullFrontalVisibilityFactor *= 0.65, HullBaseVisibilityFactor *= 0.68, IndirectVisualDetectability *= 0.7, UnderwaterFadeFactor *= 2.0, CrushDepth = -300</t>
+        </is>
+      </c>
+      <c r="T7" s="8" t="inlineStr">
+        <is>
+          <t>Entities/</t>
+        </is>
+      </c>
+      <c r="U7" s="1" t="n"/>
+      <c r="V7" s="1" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:S12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -505,780 +1096,780 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>/</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>Tags</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>Unlock date</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>Max Health</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>Durability (%)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>Design Pressure - Exterior (atm)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>Pressure Durability - Exterior</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>Design Pressure - Interior (atm)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="9" t="inlineStr">
         <is>
           <t>Pressure Durability - Interior</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="9" t="inlineStr">
         <is>
           <t>Repair Time</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="9" t="inlineStr">
         <is>
           <t>Replacement Parts</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="9" t="inlineStr">
         <is>
           <t>Dmg Dist Reduction</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="9" t="inlineStr">
         <is>
           <t>Mass</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" s="9" t="inlineStr">
         <is>
           <t>Stack Limit</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" s="9" t="inlineStr">
         <is>
           <t>Parameters</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Uses</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="R1" s="10" t="inlineStr">
         <is>
           <t>Sandbox Class</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="S1" s="10" t="inlineStr">
         <is>
           <t>Equip Sound Effect</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Accumulators I</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Accumulators, Electric Engines Upgrade</t>
         </is>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="11" t="n">
         <v>8000</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="12" t="n">
         <v>14246</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="4" t="n">
+      <c r="F2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="L2" s="7" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="M2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O2" s="4" t="n">
+      <c r="L2" s="14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="P2" s="8" t="inlineStr">
+      <c r="P2" s="15" t="inlineStr">
         <is>
           <t>EnergyCapacityGain=250%</t>
         </is>
       </c>
-      <c r="Q2" s="4" t="inlineStr">
+      <c r="Q2" s="11" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="R2" s="9" t="n"/>
-      <c r="S2" s="9" t="n"/>
+      <c r="R2" s="1" t="n"/>
+      <c r="S2" s="1" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Accumulators II</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Accumulators, Electric Engines Upgrade</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="11" t="n">
         <v>16000</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="12" t="n">
         <v>14246</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="4" t="n">
+      <c r="F3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="L3" s="7" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O3" s="4" t="n">
+      <c r="L3" s="14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="P3" s="8" t="inlineStr">
+      <c r="P3" s="15" t="inlineStr">
         <is>
           <t>EnergyCapacityGain=500%</t>
         </is>
       </c>
-      <c r="Q3" s="4" t="inlineStr">
+      <c r="Q3" s="11" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="R3" s="9" t="n"/>
-      <c r="S3" s="9" t="n"/>
+      <c r="R3" s="1" t="n"/>
+      <c r="S3" s="1" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Accumulators III</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Accumulators, Electric Engines Upgrade</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="11" t="n">
         <v>24000</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="12" t="n">
         <v>14246</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="4" t="n">
+      <c r="F4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="L4" s="7" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O4" s="4" t="n">
+      <c r="L4" s="14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="P4" s="8" t="inlineStr">
+      <c r="P4" s="15" t="inlineStr">
         <is>
           <t>EnergyCapacityGain=750%</t>
         </is>
       </c>
-      <c r="Q4" s="4" t="inlineStr">
+      <c r="Q4" s="11" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="R4" s="9" t="n"/>
-      <c r="S4" s="9" t="n"/>
+      <c r="R4" s="1" t="n"/>
+      <c r="S4" s="1" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Trim Pump</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Trim Pump</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="10" t="n">
+      <c r="C5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="16" t="n">
         <v>14246</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="13" t="n">
         <v>0.5</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G5" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="H5" s="13" t="n">
         <v>0.8</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="I5" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="J5" s="13" t="n">
         <v>0.25</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="K5" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="L5" s="7" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="M5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O5" s="4" t="n">
+      <c r="L5" s="14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="P5" s="8" t="inlineStr">
+      <c r="P5" s="15" t="inlineStr">
         <is>
           <t>LitresPerSecond = 0.06, Noise = 0.15, EnergyUsage = 2e-05</t>
         </is>
       </c>
-      <c r="Q5" s="4" t="n"/>
-      <c r="R5" s="9" t="n"/>
-      <c r="S5" s="9" t="n"/>
+      <c r="Q5" s="11" t="n"/>
+      <c r="R5" s="1" t="n"/>
+      <c r="S5" s="1" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Trim Pump Type II</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Trim Pump Type II</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="10" t="n">
+      <c r="C6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="16" t="n">
         <v>14246</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="13" t="n">
         <v>0.5</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G6" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="H6" s="13" t="n">
         <v>0.8</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="I6" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="J6" s="6" t="n">
+      <c r="J6" s="13" t="n">
         <v>0.25</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="K6" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="L6" s="7" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O6" s="4" t="n">
+      <c r="L6" s="14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="P6" s="8" t="inlineStr">
+      <c r="P6" s="15" t="inlineStr">
         <is>
           <t>LitresPerSecond = 0.06, Noise = 0.15, EnergyUsage = 2e-05</t>
         </is>
       </c>
-      <c r="Q6" s="4" t="n"/>
-      <c r="R6" s="9" t="n"/>
-      <c r="S6" s="9" t="n"/>
+      <c r="Q6" s="11" t="n"/>
+      <c r="R6" s="1" t="n"/>
+      <c r="S6" s="1" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Depth Steers Station</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="10" t="n">
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="16" t="n">
         <v>14246</v>
       </c>
-      <c r="E7" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="6" t="n">
+      <c r="E7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="13" t="n">
         <v>0.6</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="G7" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="H7" s="13" t="n">
         <v>0.7</v>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="I7" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="J7" s="6" t="n">
+      <c r="J7" s="13" t="n">
         <v>0.25</v>
       </c>
-      <c r="K7" s="4" t="n">
+      <c r="K7" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="L7" s="7" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="4" t="n">
+      <c r="L7" s="14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="O7" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P7" s="8" t="inlineStr">
+      <c r="O7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="P7" s="15" t="inlineStr">
         <is>
           <t>Noise = 0.009, EnergyUsage = 0.001</t>
         </is>
       </c>
-      <c r="Q7" s="4" t="n"/>
-      <c r="R7" s="9" t="n"/>
-      <c r="S7" s="9" t="n"/>
+      <c r="Q7" s="11" t="n"/>
+      <c r="R7" s="1" t="n"/>
+      <c r="S7" s="1" t="n"/>
     </row>
     <row r="8" ht="29.5" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Diesel Engines</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Engines, Diesel Engines</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="10" t="n">
+      <c r="C8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="16" t="n">
         <v>14246</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="F8" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="G8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="4" t="n">
+      <c r="G8" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="J8" s="6" t="n">
+      <c r="J8" s="13" t="n">
         <v>0.8</v>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="K8" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="L8" s="7" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" s="4" t="n">
+      <c r="L8" s="14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="P8" s="8" t="inlineStr">
+      <c r="P8" s="15" t="inlineStr">
         <is>
           <t>/Velocity +1, Noise = 0.7, FuelUsage = 1.0, EnergyUsage = -10, SmokeVisibility = 0.25, MaxGearChangeDelay = 7</t>
         </is>
       </c>
-      <c r="Q8" s="4" t="n"/>
-      <c r="R8" s="9" t="n"/>
-      <c r="S8" s="9" t="n"/>
+      <c r="Q8" s="11" t="n"/>
+      <c r="R8" s="1" t="n"/>
+      <c r="S8" s="1" t="n"/>
     </row>
     <row r="9" ht="29.5" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Diesel Engines IIA</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Engines, Diesel Engines IIA</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="10" t="n">
+      <c r="C9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="16" t="n">
         <v>14246</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="G9" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="4" t="n">
+      <c r="G9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="J9" s="6" t="n">
+      <c r="J9" s="13" t="n">
         <v>0.8</v>
       </c>
-      <c r="K9" s="4" t="n">
+      <c r="K9" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="L9" s="7" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="M9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O9" s="4" t="n">
+      <c r="L9" s="14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="P9" s="8" t="inlineStr">
+      <c r="P9" s="15" t="inlineStr">
         <is>
           <t>/Velocity +1, Noise = 0.35, FuelUsage = 1.0, EnergyUsage = -10, SmokeVisibility = 0.25, MaxGearChangeDelay = 7</t>
         </is>
       </c>
-      <c r="Q9" s="4" t="n"/>
-      <c r="R9" s="9" t="n"/>
-      <c r="S9" s="9" t="n"/>
+      <c r="Q9" s="11" t="n"/>
+      <c r="R9" s="1" t="n"/>
+      <c r="S9" s="1" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Electric Engines</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Engines, Electric Engines</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="10" t="n">
+      <c r="C10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="16" t="n">
         <v>14246</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="F10" s="13" t="n">
         <v>0.6</v>
       </c>
-      <c r="G10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="4" t="n">
+      <c r="G10" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="L10" s="7" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" s="4" t="n">
+      <c r="L10" s="14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="P10" s="8" t="inlineStr">
+      <c r="P10" s="15" t="inlineStr">
         <is>
           <t>/Velocity +1, Noise = 0.52, FuelUsage = 0.0, EnergyUsage = 3.5e-06, MaxGearChangeDelay = 7</t>
         </is>
       </c>
-      <c r="Q10" s="4" t="n"/>
-      <c r="R10" s="9" t="n"/>
-      <c r="S10" s="9" t="n"/>
+      <c r="Q10" s="11" t="n"/>
+      <c r="R10" s="1" t="n"/>
+      <c r="S10" s="1" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Electric Engines IIA</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Engines, Electric Engines IIA</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="10" t="n">
+      <c r="C11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="16" t="n">
         <v>14246</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="13" t="n">
         <v>0.6</v>
       </c>
-      <c r="G11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="4" t="n">
+      <c r="G11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="L11" s="7" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="M11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O11" s="4" t="n">
+      <c r="L11" s="14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O11" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="P11" s="8" t="inlineStr">
+      <c r="P11" s="15" t="inlineStr">
         <is>
           <t>/Velocity +1, Noise = 0.26, FuelUsage = 0.0, EnergyUsage = 3.5e-06, MaxGearChangeDelay = 7</t>
         </is>
       </c>
-      <c r="Q11" s="4" t="n"/>
-      <c r="R11" s="9" t="n"/>
-      <c r="S11" s="9" t="n"/>
+      <c r="Q11" s="11" t="n"/>
+      <c r="R11" s="1" t="n"/>
+      <c r="S11" s="1" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Gyrocompass</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Gyrocompass</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="10" t="n">
+      <c r="C12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="16" t="n">
         <v>14246</v>
       </c>
-      <c r="E12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="4" t="n">
+      <c r="E12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="L12" s="7" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="M12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O12" s="4" t="n">
+      <c r="L12" s="14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="P12" s="8" t="inlineStr">
+      <c r="P12" s="15" t="inlineStr">
         <is>
           <t>Noise = 0.006, EnergyUsage = 1.5e-06, NavigationImprovement = 0.4, NavigationTablePerformance = 3.0</t>
         </is>
       </c>
-      <c r="Q12" s="4" t="n"/>
-      <c r="R12" s="9" t="n"/>
-      <c r="S12" s="9" t="n"/>
+      <c r="Q12" s="11" t="n"/>
+      <c r="R12" s="1" t="n"/>
+      <c r="S12" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Support Type IX DLC speed cap
</commit_message>
<xml_diff>
--- a/LongSubmerged10x/Data Sheets/Entities.xlsx
+++ b/LongSubmerged10x/Data Sheets/Entities.xlsx
@@ -17,11 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,6 +64,12 @@
       <charset val="1"/>
       <family val="2"/>
       <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="238"/>
+      <family val="2"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -121,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -150,7 +155,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -162,7 +167,25 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -530,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:V10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.54296875" customWidth="1" min="1" max="1"/>
@@ -1059,6 +1082,225 @@
       </c>
       <c r="U7" s="1" t="n"/>
       <c r="V7" s="1" t="n"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Type IXA (Player)</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Submarine</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>769</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>871</v>
+      </c>
+      <c r="F8" s="17" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="H8" s="17" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="I8" s="18" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J8" s="19" t="n"/>
+      <c r="K8" s="17" t="n">
+        <v>24910</v>
+      </c>
+      <c r="L8" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="M8" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="O8" s="17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>7500</v>
+      </c>
+      <c r="Q8" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="S8" s="20" t="inlineStr">
+        <is>
+          <t>Observation Spot/SightRange = 8500, Observation Spot/GroupSightRange = 13, AreaSize = 7.5, SpawnSpacing = 300, HullFrontalVisibilityFactor *= 0.65, HullBaseVisibilityFactor *= 0.68, IndirectVisualDetectability *= 0.7, UnderwaterFadeFactor *= 2.0, CrushDepth = -230</t>
+        </is>
+      </c>
+      <c r="T8" s="20" t="inlineStr">
+        <is>
+          <t>Entities/</t>
+        </is>
+      </c>
+      <c r="U8" s="17" t="n"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Type IXC (Player)</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Submarine</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="D9" s="17" t="n">
+        <v>769</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>871</v>
+      </c>
+      <c r="F9" s="17" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="G9" s="17" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="H9" s="17" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="I9" s="18" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J9" s="19" t="n"/>
+      <c r="K9" s="17" t="n">
+        <v>24910</v>
+      </c>
+      <c r="L9" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="M9" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="N9" s="17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="O9" s="17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>7500</v>
+      </c>
+      <c r="Q9" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="S9" s="20" t="inlineStr">
+        <is>
+          <t>Observation Spot/SightRange = 8500, Observation Spot/GroupSightRange = 13, AreaSize = 7.5, SpawnSpacing = 300, HullFrontalVisibilityFactor *= 0.65, HullBaseVisibilityFactor *= 0.68, IndirectVisualDetectability *= 0.7, UnderwaterFadeFactor *= 2.0, CrushDepth = -230</t>
+        </is>
+      </c>
+      <c r="T9" s="20" t="inlineStr">
+        <is>
+          <t>Entities/</t>
+        </is>
+      </c>
+      <c r="U9" s="17" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>Type IXC40 (Player)</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Submarine</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>769</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>871</v>
+      </c>
+      <c r="F10" s="17" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="G10" s="17" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="H10" s="17" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="I10" s="18" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J10" s="19" t="n"/>
+      <c r="K10" s="17" t="n">
+        <v>24910</v>
+      </c>
+      <c r="L10" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="M10" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="O10" s="17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>7500</v>
+      </c>
+      <c r="Q10" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="S10" s="20" t="inlineStr">
+        <is>
+          <t>Observation Spot/SightRange = 8500, Observation Spot/GroupSightRange = 13, AreaSize = 7.5, SpawnSpacing = 300, HullFrontalVisibilityFactor *= 0.65, HullBaseVisibilityFactor *= 0.68, IndirectVisualDetectability *= 0.7, UnderwaterFadeFactor *= 2.0, CrushDepth = -230</t>
+        </is>
+      </c>
+      <c r="T10" s="20" t="inlineStr">
+        <is>
+          <t>Entities/</t>
+        </is>
+      </c>
+      <c r="U10" s="17" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1206,7 +1448,7 @@
       <c r="C2" s="11" t="n">
         <v>8000</v>
       </c>
-      <c r="D2" s="12" t="n">
+      <c r="D2" s="21" t="n">
         <v>14246</v>
       </c>
       <c r="E2" s="11" t="n">
@@ -1271,7 +1513,7 @@
       <c r="C3" s="11" t="n">
         <v>16000</v>
       </c>
-      <c r="D3" s="12" t="n">
+      <c r="D3" s="21" t="n">
         <v>14246</v>
       </c>
       <c r="E3" s="11" t="n">
@@ -1336,7 +1578,7 @@
       <c r="C4" s="11" t="n">
         <v>24000</v>
       </c>
-      <c r="D4" s="12" t="n">
+      <c r="D4" s="21" t="n">
         <v>14246</v>
       </c>
       <c r="E4" s="11" t="n">
@@ -1401,7 +1643,7 @@
       <c r="C5" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="16" t="n">
+      <c r="D5" s="22" t="n">
         <v>14246</v>
       </c>
       <c r="E5" s="11" t="n">
@@ -1462,7 +1704,7 @@
       <c r="C6" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="16" t="n">
+      <c r="D6" s="22" t="n">
         <v>14246</v>
       </c>
       <c r="E6" s="11" t="n">
@@ -1519,7 +1761,7 @@
       <c r="C7" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="22" t="n">
         <v>14246</v>
       </c>
       <c r="E7" s="11" t="n">
@@ -1580,7 +1822,7 @@
       <c r="C8" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D8" s="22" t="n">
         <v>14246</v>
       </c>
       <c r="E8" s="11" t="n">
@@ -1641,7 +1883,7 @@
       <c r="C9" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="22" t="n">
         <v>14246</v>
       </c>
       <c r="E9" s="11" t="n">
@@ -1702,7 +1944,7 @@
       <c r="C10" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="16" t="n">
+      <c r="D10" s="22" t="n">
         <v>14246</v>
       </c>
       <c r="E10" s="11" t="n">
@@ -1763,7 +2005,7 @@
       <c r="C11" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="22" t="n">
         <v>14246</v>
       </c>
       <c r="E11" s="11" t="n">
@@ -1824,7 +2066,7 @@
       <c r="C12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="16" t="n">
+      <c r="D12" s="22" t="n">
         <v>14246</v>
       </c>
       <c r="E12" s="11" t="n">

</xml_diff>

<commit_message>
Fix fast speed propulsion and battery recharge
</commit_message>
<xml_diff>
--- a/LongSubmerged10x/Data Sheets/Entities.xlsx
+++ b/LongSubmerged10x/Data Sheets/Entities.xlsx
@@ -1313,7 +1313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:S10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="47.54296875" customWidth="1" min="1" max="1"/>
@@ -1808,15 +1808,15 @@
       <c r="R7" s="1" t="n"/>
       <c r="S7" s="1" t="n"/>
     </row>
-    <row r="8" ht="29.5" customHeight="1">
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Diesel Engines</t>
+          <t>Electric Engines</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Engines, Diesel Engines</t>
+          <t>Engines, Electric Engines</t>
         </is>
       </c>
       <c r="C8" s="11" t="n">
@@ -1829,7 +1829,7 @@
         <v>4</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="G8" s="11" t="n">
         <v>1</v>
@@ -1838,10 +1838,10 @@
         <v>0</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="J8" s="13" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="K8" s="11" t="n">
         <v>60</v>
@@ -1862,22 +1862,22 @@
       </c>
       <c r="P8" s="15" t="inlineStr">
         <is>
-          <t>/Velocity +1, Noise = 0.7, FuelUsage = 1.0, EnergyUsage = -10, SmokeVisibility = 0.25, MaxGearChangeDelay = 7</t>
+          <t>/Velocity +1, Noise = 0.52, FuelUsage = 0.0, EnergyUsage = 3.5e-06, MaxGearChangeDelay = 7</t>
         </is>
       </c>
       <c r="Q8" s="11" t="n"/>
       <c r="R8" s="1" t="n"/>
       <c r="S8" s="1" t="n"/>
     </row>
-    <row r="9" ht="29.5" customHeight="1">
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>Diesel Engines IIA</t>
+          <t>Electric Engines IIA</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Engines, Diesel Engines IIA</t>
+          <t>Engines, Electric Engines IIA</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
@@ -1890,7 +1890,7 @@
         <v>4</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="G9" s="11" t="n">
         <v>1</v>
@@ -1899,10 +1899,10 @@
         <v>0</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="J9" s="13" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="K9" s="11" t="n">
         <v>60</v>
@@ -1923,7 +1923,7 @@
       </c>
       <c r="P9" s="15" t="inlineStr">
         <is>
-          <t>/Velocity +1, Noise = 0.35, FuelUsage = 1.0, EnergyUsage = -10, SmokeVisibility = 0.25, MaxGearChangeDelay = 7</t>
+          <t>/Velocity +1, Noise = 0.26, FuelUsage = 0.0, EnergyUsage = 3.5e-06, MaxGearChangeDelay = 7</t>
         </is>
       </c>
       <c r="Q9" s="11" t="n"/>
@@ -1933,12 +1933,12 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Electric Engines</t>
+          <t>Gyrocompass</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Engines, Electric Engines</t>
+          <t>Gyrocompass</t>
         </is>
       </c>
       <c r="C10" s="11" t="n">
@@ -1948,10 +1948,10 @@
         <v>14246</v>
       </c>
       <c r="E10" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="G10" s="11" t="n">
         <v>1</v>
@@ -1984,134 +1984,12 @@
       </c>
       <c r="P10" s="15" t="inlineStr">
         <is>
-          <t>/Velocity +1, Noise = 0.52, FuelUsage = 0.0, EnergyUsage = 3.5e-06, MaxGearChangeDelay = 7</t>
+          <t>Noise = 0.006, EnergyUsage = 1.5e-06, NavigationImprovement = 0.4, NavigationTablePerformance = 3.0</t>
         </is>
       </c>
       <c r="Q10" s="11" t="n"/>
       <c r="R10" s="1" t="n"/>
       <c r="S10" s="1" t="n"/>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>Electric Engines IIA</t>
-        </is>
-      </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>Engines, Electric Engines IIA</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="22" t="n">
-        <v>14246</v>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="F11" s="13" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G11" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="11" t="n">
-        <v>60</v>
-      </c>
-      <c r="L11" s="14" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="M11" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="O11" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="P11" s="15" t="inlineStr">
-        <is>
-          <t>/Velocity +1, Noise = 0.26, FuelUsage = 0.0, EnergyUsage = 3.5e-06, MaxGearChangeDelay = 7</t>
-        </is>
-      </c>
-      <c r="Q11" s="11" t="n"/>
-      <c r="R11" s="1" t="n"/>
-      <c r="S11" s="1" t="n"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>Gyrocompass</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>Gyrocompass</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="22" t="n">
-        <v>14246</v>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="11" t="n">
-        <v>60</v>
-      </c>
-      <c r="L12" s="14" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="M12" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="O12" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="P12" s="15" t="inlineStr">
-        <is>
-          <t>Noise = 0.006, EnergyUsage = 1.5e-06, NavigationImprovement = 0.4, NavigationTablePerformance = 3.0</t>
-        </is>
-      </c>
-      <c r="Q12" s="11" t="n"/>
-      <c r="R12" s="1" t="n"/>
-      <c r="S12" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>